<commit_message>
Fotos de directiva, mascota, jugadores y galería por serie
- Directiva: foto de Feliciciano Barra y Daniel Muñoz
- Mascota: foto de Chocolo
- Jugadores: fotos nuevas para Sr35 (Rodrigo Catalán, Jonathan Vasquez,
  Jerson Constanzo, Juan Pablo Martínez, Carlos Navarro, Christian
  López, Francisco Araya, Juan Carlos Catalán, Ariel Nicolao, Jonathan
  Ortega) y actualiza 3 fotos existentes
- Galería: fotos históricas (Campeón 1973, Población San Rafael,
  Plantel Histórico) y fotos por serie de Senior 35 y Senior 45
  (plantel + partido vs Jorge Toro)
- Calendario: resultados y próximos partidos actualizados
- Ignora los archivos temporales de bloqueo de Excel (~$*.xlsx)
</commit_message>
<xml_diff>
--- a/data/calendario.xlsx
+++ b/data/calendario.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marce\Proyectos\juventud-san-rafael\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F743BFB-38CD-4F6D-AAF1-B2904091A176}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBA2E21A-9610-4015-842C-CE9B8F3B36D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="39">
   <si>
     <t>fecha</t>
   </si>
@@ -104,6 +104,39 @@
   </si>
   <si>
     <t>Complejo Deportivo Las Rosas - Cancha 1</t>
+  </si>
+  <si>
+    <t>2 - 1</t>
+  </si>
+  <si>
+    <t>1 - 5</t>
+  </si>
+  <si>
+    <t>2 - 3</t>
+  </si>
+  <si>
+    <t>No informado</t>
+  </si>
+  <si>
+    <t>2026-09-04</t>
+  </si>
+  <si>
+    <t>2026-09-06</t>
+  </si>
+  <si>
+    <t>15:00</t>
+  </si>
+  <si>
+    <t>Senior 60</t>
+  </si>
+  <si>
+    <t>Complejo Deportivo Las Rosas</t>
+  </si>
+  <si>
+    <t>No Informado</t>
+  </si>
+  <si>
+    <t>Juventud Nueva Estrella</t>
   </si>
 </sst>
 </file>
@@ -444,7 +477,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" style="1" customWidth="1"/>
@@ -453,7 +486,7 @@
     <col min="4" max="4" width="25" customWidth="1"/>
     <col min="5" max="5" width="11" customWidth="1"/>
     <col min="6" max="6" width="36.33203125" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="7" max="7" width="14.33203125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -475,7 +508,7 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
@@ -498,6 +531,9 @@
       <c r="F2" t="s">
         <v>27</v>
       </c>
+      <c r="G2" s="1" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -518,6 +554,9 @@
       <c r="F3" t="s">
         <v>27</v>
       </c>
+      <c r="G3" s="1" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
@@ -538,6 +577,9 @@
       <c r="F4" t="s">
         <v>27</v>
       </c>
+      <c r="G4" s="1" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -558,6 +600,9 @@
       <c r="F5" t="s">
         <v>27</v>
       </c>
+      <c r="G5" s="1" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
@@ -578,6 +623,9 @@
       <c r="F6" t="s">
         <v>27</v>
       </c>
+      <c r="G6" s="1" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
@@ -598,6 +646,9 @@
       <c r="F7" t="s">
         <v>27</v>
       </c>
+      <c r="G7" s="1" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -618,6 +669,9 @@
       <c r="F8" t="s">
         <v>27</v>
       </c>
+      <c r="G8" s="1" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
@@ -637,6 +691,209 @@
       </c>
       <c r="F9" t="s">
         <v>27</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" t="s">
+        <v>26</v>
+      </c>
+      <c r="F11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" t="s">
+        <v>38</v>
+      </c>
+      <c r="E12" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" t="s">
+        <v>38</v>
+      </c>
+      <c r="E13" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" t="s">
+        <v>38</v>
+      </c>
+      <c r="E14" t="s">
+        <v>26</v>
+      </c>
+      <c r="F14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" t="s">
+        <v>26</v>
+      </c>
+      <c r="F15" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" t="s">
+        <v>38</v>
+      </c>
+      <c r="E16" t="s">
+        <v>26</v>
+      </c>
+      <c r="F16" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" t="s">
+        <v>38</v>
+      </c>
+      <c r="E17" t="s">
+        <v>26</v>
+      </c>
+      <c r="F17" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" t="s">
+        <v>38</v>
+      </c>
+      <c r="E18" t="s">
+        <v>26</v>
+      </c>
+      <c r="F18" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C19" t="s">
+        <v>35</v>
+      </c>
+      <c r="D19" t="s">
+        <v>37</v>
+      </c>
+      <c r="E19" t="s">
+        <v>26</v>
+      </c>
+      <c r="F19" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualiza resultado del partido Senior 60 vs Jorge Toro
</commit_message>
<xml_diff>
--- a/data/calendario.xlsx
+++ b/data/calendario.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marce\Proyectos\juventud-san-rafael\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBA2E21A-9610-4015-842C-CE9B8F3B36D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBB9F26F-6484-4714-BEF1-1D635170D171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="39">
   <si>
     <t>fecha</t>
   </si>
@@ -707,13 +707,16 @@
         <v>35</v>
       </c>
       <c r="D10" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="E10" t="s">
         <v>26</v>
       </c>
       <c r="F10" t="s">
-        <v>36</v>
+        <v>37</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>